<commit_message>
Nueva columna indice de eficiencia en la terminación
</commit_message>
<xml_diff>
--- a/Contexto/MatrizSeguimientoEvaluacion_20260609_1833.xlsx
+++ b/Contexto/MatrizSeguimientoEvaluacion_20260609_1833.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://departamentodesucre.sharepoint.com/sites/SeguimientoRegalas/Documentos compartidos/Regalías/GESTION Y SEGUIMIENTO SGR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Donaldo Acosta\Documents\MEGA\Estudio\python\Consolidacion Regalias\Contexto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{6976D422-6619-4961-9443-0A3B7DFE6DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9B1D70B-C6F5-4423-8656-01DBF6787A28}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E8E490-E475-4F19-9B42-6A17336A36BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MatrizSeguimientoEvaluacion" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="1016">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2025" uniqueCount="1016">
   <si>
     <t>DATOS GENERALES</t>
   </si>
@@ -3348,7 +3348,42 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Roboto"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3467,7 +3502,7 @@
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="FECHA DE SUSCRIPCIÓN DEL PRIMER CONTRATO"/>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="FECHA ACTA INICIO"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="HORIZONTE DEL PROYECTO"/>
-    <tableColumn id="54" xr3:uid="{5E233D81-7827-4B0C-BCCB-CBA1ADD4E332}" name="FECHA DE SUSPENSIÓN DEL CONTRATO " dataDxfId="1"/>
+    <tableColumn id="54" xr3:uid="{5E233D81-7827-4B0C-BCCB-CBA1ADD4E332}" name="FECHA DE SUSPENSIÓN DEL CONTRATO " dataDxfId="2"/>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="FECHA DE FINALIZACIÓN"/>
     <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="FECHA EN LA QUE PASO A ESTADO PARA CIERRE"/>
     <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="FECHA DE CORTE GESPROY"/>
@@ -3487,7 +3522,7 @@
     <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="CALIFICACIÓN CALIDAD INFORMACIÓN"/>
     <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="COLUMNA APOYO 2"/>
     <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="CALIFICACIÓN EJECUCIÓN DEL PROYECTO"/>
-    <tableColumn id="53" xr3:uid="{7C812041-A764-423A-8F04-DFE8AC012AC3}" name="ÍNDICE DE EFICIENCIA EN LA TERMINACIÓN" dataDxfId="0"/>
+    <tableColumn id="53" xr3:uid="{7C812041-A764-423A-8F04-DFE8AC012AC3}" name="ÍNDICE DE EFICIENCIA EN LA TERMINACIÓN" dataDxfId="1"/>
     <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="COMENTARIOS CALIFICACIÓN"/>
     <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="RESPONSABLE CARGUE EN GESPROY"/>
     <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="MUNICIPIOS"/>
@@ -3497,9 +3532,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="OtrosEjecutoresDescentralizadas" displayName="OtrosEjecutoresDescentralizadas" ref="A2:AO18" totalsRowShown="0">
-  <autoFilter ref="A2:AO18" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="OtrosEjecutoresDescentralizadas" displayName="OtrosEjecutoresDescentralizadas" ref="A2:AP18" totalsRowShown="0">
+  <autoFilter ref="A2:AP18" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="42">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="BPIN"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="EJECUTOR"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="NOMBRE DEL PROYECTO"/>
@@ -3539,6 +3574,7 @@
     <tableColumn id="37" xr3:uid="{00000000-0010-0000-0100-000025000000}" name="CALIFICACIÓN CALIDAD INFORMACIÓN"/>
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0100-000026000000}" name="COLUMNA APOYO 2"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0100-000027000000}" name="CALIFICACIÓN EJECUCIÓN DEL PROYECTO"/>
+    <tableColumn id="42" xr3:uid="{8C83C1C6-E74B-4242-83E7-659AAED76935}" name="ÍNDICE DE EFICIENCIA EN LA TERMINACIÓN" dataDxfId="0"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0100-000028000000}" name="COMENTARIOS CALIFICACIÓN"/>
     <tableColumn id="41" xr3:uid="{00000000-0010-0000-0100-000029000000}" name="MUNICIPIOS"/>
   </tableColumns>
@@ -12819,17 +12855,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AO18"/>
+  <dimension ref="A1:AP18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="31" width="25.6640625" customWidth="1"/>
     <col min="32" max="32" width="25.6640625" hidden="1" customWidth="1"/>
     <col min="33" max="37" width="25.6640625" customWidth="1"/>
     <col min="38" max="38" width="25.6640625" hidden="1" customWidth="1"/>
-    <col min="39" max="41" width="25.6640625" customWidth="1"/>
+    <col min="39" max="42" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:42" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -12877,8 +12913,9 @@
       <c r="AM1" s="7"/>
       <c r="AN1" s="7"/>
       <c r="AO1" s="7"/>
+      <c r="AP1" s="7"/>
     </row>
-    <row r="2" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -12997,13 +13034,16 @@
         <v>51</v>
       </c>
       <c r="AN2" s="1" t="s">
+        <v>1010</v>
+      </c>
+      <c r="AO2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AO2" s="3" t="s">
+      <c r="AP2" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>509</v>
       </c>
@@ -13105,14 +13145,15 @@
         <f t="shared" ref="AM3:AM18" si="5">IFERROR(IF($G3="CONTRATADO EN EJECUCIÓN",IF(AND(ISNUMBER($X3),ISNUMBER($Z3),$X3&lt;$Z3),0,IF($AH3&gt;=1,(IFERROR(IF(ISNUMBER($AJ3),($AD3*0.4+$AE3*0.2+$AG3*0.4),""),""))*$AL3/100,IFERROR(IF(ISNUMBER($AJ3),($AD3*0.4+$AE3*0.2+$AG3*0.4),""),""))),IF($G3="CONTRATADO SIN ACTA DE INICIO",IF(AND($Z3-$V3&gt;=0,$Z3-$V3&lt;=30),100,0),"")),"")</f>
         <v/>
       </c>
-      <c r="AN3" s="4" t="s">
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="AO3" s="4" t="s">
+      <c r="AP3" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>516</v>
       </c>
@@ -13214,14 +13255,15 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AN4" s="4" t="s">
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="AO4" s="4" t="s">
+      <c r="AP4" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>520</v>
       </c>
@@ -13329,14 +13371,15 @@
         <f t="shared" si="5"/>
         <v>75</v>
       </c>
-      <c r="AN5" s="4" t="s">
+      <c r="AN5" s="4"/>
+      <c r="AO5" s="4" t="s">
         <v>525</v>
       </c>
-      <c r="AO5" s="4" t="s">
+      <c r="AP5" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>526</v>
       </c>
@@ -13446,14 +13489,15 @@
         <f t="shared" si="5"/>
         <v>50</v>
       </c>
-      <c r="AN6" s="4" t="s">
+      <c r="AN6" s="4"/>
+      <c r="AO6" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="AO6" s="4" t="s">
+      <c r="AP6" s="4" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="7" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>532</v>
       </c>
@@ -13563,14 +13607,15 @@
         <f t="shared" si="5"/>
         <v>50</v>
       </c>
-      <c r="AN7" s="4" t="s">
+      <c r="AN7" s="4"/>
+      <c r="AO7" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="AO7" s="4" t="s">
+      <c r="AP7" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>536</v>
       </c>
@@ -13672,14 +13717,15 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AN8" s="4" t="s">
+      <c r="AN8" s="4"/>
+      <c r="AO8" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="AO8" s="4" t="s">
+      <c r="AP8" s="4" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="9" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>540</v>
       </c>
@@ -13789,14 +13835,15 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AN9" s="4" t="s">
+      <c r="AN9" s="4"/>
+      <c r="AO9" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="AO9" s="4" t="s">
+      <c r="AP9" s="4" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="10" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>545</v>
       </c>
@@ -13905,11 +13952,12 @@
         <v>100</v>
       </c>
       <c r="AN10" s="4"/>
-      <c r="AO10" s="4" t="s">
+      <c r="AO10" s="4"/>
+      <c r="AP10" s="4" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="11" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>548</v>
       </c>
@@ -14020,11 +14068,12 @@
         <v>60</v>
       </c>
       <c r="AN11" s="4"/>
-      <c r="AO11" s="4" t="s">
+      <c r="AO11" s="4"/>
+      <c r="AP11" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>551</v>
       </c>
@@ -14134,14 +14183,15 @@
         <f t="shared" si="5"/>
         <v>90</v>
       </c>
-      <c r="AN12" s="4" t="s">
+      <c r="AN12" s="4"/>
+      <c r="AO12" s="4" t="s">
         <v>555</v>
       </c>
-      <c r="AO12" s="4" t="s">
+      <c r="AP12" s="4" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="13" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>557</v>
       </c>
@@ -14250,11 +14300,12 @@
         <v/>
       </c>
       <c r="AN13" s="4"/>
-      <c r="AO13" s="4" t="s">
+      <c r="AO13" s="4"/>
+      <c r="AP13" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>560</v>
       </c>
@@ -14365,11 +14416,12 @@
         <v>30</v>
       </c>
       <c r="AN14" s="4"/>
-      <c r="AO14" s="4" t="s">
+      <c r="AO14" s="4"/>
+      <c r="AP14" s="4" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="15" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>564</v>
       </c>
@@ -14478,11 +14530,12 @@
         <v>100</v>
       </c>
       <c r="AN15" s="4"/>
-      <c r="AO15" s="4" t="s">
+      <c r="AO15" s="4"/>
+      <c r="AP15" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="16" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>568</v>
       </c>
@@ -14591,11 +14644,12 @@
         <v>0</v>
       </c>
       <c r="AN16" s="4"/>
-      <c r="AO16" s="4" t="s">
+      <c r="AO16" s="4"/>
+      <c r="AP16" s="4" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="17" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>571</v>
       </c>
@@ -14696,11 +14750,12 @@
         <v>40</v>
       </c>
       <c r="AN17" s="4"/>
-      <c r="AO17" s="4" t="s">
+      <c r="AO17" s="4"/>
+      <c r="AP17" s="4" t="s">
         <v>574</v>
       </c>
     </row>
-    <row r="18" spans="1:41" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>575</v>
       </c>
@@ -14799,7 +14854,8 @@
         <v/>
       </c>
       <c r="AN18" s="4"/>
-      <c r="AO18" s="4" t="s">
+      <c r="AO18" s="4"/>
+      <c r="AP18" s="4" t="s">
         <v>580</v>
       </c>
     </row>
@@ -14807,7 +14863,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="O1:AH1"/>
-    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="AI1:AP1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -20498,9 +20554,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20648,19 +20707,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65E8F416-0DD0-4166-9ACF-D00744BB634B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B86AA879-F6E4-4512-AC7A-AB9CD1300842}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -20684,9 +20739,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B86AA879-F6E4-4512-AC7A-AB9CD1300842}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65E8F416-0DD0-4166-9ACF-D00744BB634B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>